<commit_message>
Combined data and metadata
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aditpatel/Desktop/MSU/Spring 2026/Intro to AI/Project 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264742EF-284A-0B44-AA7F-8E9D054FAE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18AE4F45-6EBA-494A-9B69-03E4B8D85199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="1700" windowWidth="27640" windowHeight="16680" xr2:uid="{B5B07997-311F-C649-8D95-3B8C8BF43D8D}"/>
+    <workbookView xWindow="4420" yWindow="1220" windowWidth="25820" windowHeight="16680" xr2:uid="{B5B07997-311F-C649-8D95-3B8C8BF43D8D}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
+    <sheet name="metadata" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="21">
   <si>
     <t>Top</t>
   </si>
@@ -32,6 +33,57 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>bottom</t>
+  </si>
+  <si>
+    <t>purple</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>navy</t>
+  </si>
+  <si>
+    <t>gray</t>
+  </si>
+  <si>
+    <t>blue</t>
+  </si>
+  <si>
+    <t>top</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>pink</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>khaki</t>
+  </si>
+  <si>
+    <t>Frequency (Score &gt;=7)</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Warmth</t>
+  </si>
+  <si>
+    <t>Formality</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Item</t>
   </si>
 </sst>
 </file>
@@ -924,28 +976,664 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>33</v>
+      </c>
+      <c r="C3">
+        <v>75</v>
+      </c>
       <c r="D3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>60</v>
+      </c>
       <c r="D4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <v>80</v>
+      </c>
       <c r="D5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>29</v>
+      </c>
+      <c r="C6">
+        <v>20</v>
+      </c>
       <c r="D6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>25</v>
+      </c>
+      <c r="B7">
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>90</v>
+      </c>
       <c r="D7">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B66A724-369A-1148-BB98-084F0ADBCFF1}">
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>8</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>9</v>
+      </c>
+      <c r="E20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24">
+        <v>4</v>
+      </c>
+      <c r="D24">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>9</v>
+      </c>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>9</v>
+      </c>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>7</v>
+      </c>
+      <c r="E28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>8</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32">
+        <v>3</v>
+      </c>
+      <c r="D32">
+        <v>3</v>
+      </c>
+      <c r="E32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33">
+        <v>3</v>
+      </c>
+      <c r="D33">
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+      <c r="D34">
+        <v>3</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more data and a new sheet that displays how many data points
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3,26 +3,33 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="1220" windowWidth="25820" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3540" yWindow="1060" windowWidth="25820" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -445,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D214"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -1518,6 +1525,1938 @@
       </c>
       <c r="D76" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>19</v>
+      </c>
+      <c r="B77" t="n">
+        <v>2</v>
+      </c>
+      <c r="C77" t="n">
+        <v>37</v>
+      </c>
+      <c r="D77" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>19</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="n">
+        <v>33</v>
+      </c>
+      <c r="D78" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>13</v>
+      </c>
+      <c r="B79" t="n">
+        <v>23</v>
+      </c>
+      <c r="C79" t="n">
+        <v>40</v>
+      </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>12</v>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="n">
+        <v>23</v>
+      </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>11</v>
+      </c>
+      <c r="B81" t="n">
+        <v>33</v>
+      </c>
+      <c r="C81" t="n">
+        <v>33</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>12</v>
+      </c>
+      <c r="B82" t="n">
+        <v>33</v>
+      </c>
+      <c r="C82" t="n">
+        <v>81</v>
+      </c>
+      <c r="D82" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>13</v>
+      </c>
+      <c r="B83" t="n">
+        <v>33</v>
+      </c>
+      <c r="C83" t="n">
+        <v>22</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>3</v>
+      </c>
+      <c r="B84" t="n">
+        <v>32</v>
+      </c>
+      <c r="C84" t="n">
+        <v>75</v>
+      </c>
+      <c r="D84" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>4</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" t="n">
+        <v>37</v>
+      </c>
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>4</v>
+      </c>
+      <c r="B86" t="n">
+        <v>29</v>
+      </c>
+      <c r="C86" t="n">
+        <v>31</v>
+      </c>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>12</v>
+      </c>
+      <c r="B87" t="n">
+        <v>24</v>
+      </c>
+      <c r="C87" t="n">
+        <v>35</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>15</v>
+      </c>
+      <c r="B88" t="n">
+        <v>31</v>
+      </c>
+      <c r="C88" t="n">
+        <v>25</v>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>27</v>
+      </c>
+      <c r="B89" t="n">
+        <v>30</v>
+      </c>
+      <c r="C89" t="n">
+        <v>69</v>
+      </c>
+      <c r="D89" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>14</v>
+      </c>
+      <c r="B90" t="n">
+        <v>29</v>
+      </c>
+      <c r="C90" t="n">
+        <v>26</v>
+      </c>
+      <c r="D90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>17</v>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" t="n">
+        <v>58</v>
+      </c>
+      <c r="D91" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>26</v>
+      </c>
+      <c r="B92" t="n">
+        <v>29</v>
+      </c>
+      <c r="C92" t="n">
+        <v>83</v>
+      </c>
+      <c r="D92" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>19</v>
+      </c>
+      <c r="B93" t="n">
+        <v>32</v>
+      </c>
+      <c r="C93" t="n">
+        <v>26</v>
+      </c>
+      <c r="D93" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>15</v>
+      </c>
+      <c r="B94" t="n">
+        <v>32</v>
+      </c>
+      <c r="C94" t="n">
+        <v>48</v>
+      </c>
+      <c r="D94" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>25</v>
+      </c>
+      <c r="B95" t="n">
+        <v>29</v>
+      </c>
+      <c r="C95" t="n">
+        <v>61</v>
+      </c>
+      <c r="D95" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>25</v>
+      </c>
+      <c r="B96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C96" t="n">
+        <v>71</v>
+      </c>
+      <c r="D96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>25</v>
+      </c>
+      <c r="B97" t="n">
+        <v>2</v>
+      </c>
+      <c r="C97" t="n">
+        <v>52</v>
+      </c>
+      <c r="D97" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>5</v>
+      </c>
+      <c r="B98" t="n">
+        <v>23</v>
+      </c>
+      <c r="C98" t="n">
+        <v>87</v>
+      </c>
+      <c r="D98" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>5</v>
+      </c>
+      <c r="B99" t="n">
+        <v>2</v>
+      </c>
+      <c r="C99" t="n">
+        <v>28</v>
+      </c>
+      <c r="D99" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>10</v>
+      </c>
+      <c r="B100" t="n">
+        <v>30</v>
+      </c>
+      <c r="C100" t="n">
+        <v>89</v>
+      </c>
+      <c r="D100" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>4</v>
+      </c>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" t="n">
+        <v>44</v>
+      </c>
+      <c r="D101" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>10</v>
+      </c>
+      <c r="B102" t="n">
+        <v>24</v>
+      </c>
+      <c r="C102" t="n">
+        <v>58</v>
+      </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>16</v>
+      </c>
+      <c r="B103" t="n">
+        <v>31</v>
+      </c>
+      <c r="C103" t="n">
+        <v>30</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>9</v>
+      </c>
+      <c r="B104" t="n">
+        <v>24</v>
+      </c>
+      <c r="C104" t="n">
+        <v>27</v>
+      </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>16</v>
+      </c>
+      <c r="B105" t="n">
+        <v>32</v>
+      </c>
+      <c r="C105" t="n">
+        <v>87</v>
+      </c>
+      <c r="D105" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>16</v>
+      </c>
+      <c r="B106" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" t="n">
+        <v>40</v>
+      </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>12</v>
+      </c>
+      <c r="B107" t="n">
+        <v>30</v>
+      </c>
+      <c r="C107" t="n">
+        <v>78</v>
+      </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>4</v>
+      </c>
+      <c r="B108" t="n">
+        <v>32</v>
+      </c>
+      <c r="C108" t="n">
+        <v>62</v>
+      </c>
+      <c r="D108" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>17</v>
+      </c>
+      <c r="B109" t="n">
+        <v>31</v>
+      </c>
+      <c r="C109" t="n">
+        <v>53</v>
+      </c>
+      <c r="D109" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>4</v>
+      </c>
+      <c r="B110" t="n">
+        <v>32</v>
+      </c>
+      <c r="C110" t="n">
+        <v>55</v>
+      </c>
+      <c r="D110" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>27</v>
+      </c>
+      <c r="B111" t="n">
+        <v>29</v>
+      </c>
+      <c r="C111" t="n">
+        <v>80</v>
+      </c>
+      <c r="D111" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>25</v>
+      </c>
+      <c r="B112" t="n">
+        <v>21</v>
+      </c>
+      <c r="C112" t="n">
+        <v>51</v>
+      </c>
+      <c r="D112" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>18</v>
+      </c>
+      <c r="B113" t="n">
+        <v>29</v>
+      </c>
+      <c r="C113" t="n">
+        <v>74</v>
+      </c>
+      <c r="D113" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>15</v>
+      </c>
+      <c r="B114" t="n">
+        <v>31</v>
+      </c>
+      <c r="C114" t="n">
+        <v>48</v>
+      </c>
+      <c r="D114" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>18</v>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" t="n">
+        <v>56</v>
+      </c>
+      <c r="D115" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>15</v>
+      </c>
+      <c r="B116" t="n">
+        <v>33</v>
+      </c>
+      <c r="C116" t="n">
+        <v>82</v>
+      </c>
+      <c r="D116" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>25</v>
+      </c>
+      <c r="B117" t="n">
+        <v>24</v>
+      </c>
+      <c r="C117" t="n">
+        <v>90</v>
+      </c>
+      <c r="D117" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>11</v>
+      </c>
+      <c r="B118" t="n">
+        <v>21</v>
+      </c>
+      <c r="C118" t="n">
+        <v>81</v>
+      </c>
+      <c r="D118" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>16</v>
+      </c>
+      <c r="B119" t="n">
+        <v>1</v>
+      </c>
+      <c r="C119" t="n">
+        <v>39</v>
+      </c>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>10</v>
+      </c>
+      <c r="B120" t="n">
+        <v>1</v>
+      </c>
+      <c r="C120" t="n">
+        <v>22</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>15</v>
+      </c>
+      <c r="B121" t="n">
+        <v>21</v>
+      </c>
+      <c r="C121" t="n">
+        <v>46</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>19</v>
+      </c>
+      <c r="B122" t="n">
+        <v>29</v>
+      </c>
+      <c r="C122" t="n">
+        <v>86</v>
+      </c>
+      <c r="D122" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>6</v>
+      </c>
+      <c r="B123" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" t="n">
+        <v>41</v>
+      </c>
+      <c r="D123" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>3</v>
+      </c>
+      <c r="B124" t="n">
+        <v>29</v>
+      </c>
+      <c r="C124" t="n">
+        <v>68</v>
+      </c>
+      <c r="D124" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>11</v>
+      </c>
+      <c r="B125" t="n">
+        <v>30</v>
+      </c>
+      <c r="C125" t="n">
+        <v>40</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>3</v>
+      </c>
+      <c r="B126" t="n">
+        <v>24</v>
+      </c>
+      <c r="C126" t="n">
+        <v>88</v>
+      </c>
+      <c r="D126" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>4</v>
+      </c>
+      <c r="B127" t="n">
+        <v>33</v>
+      </c>
+      <c r="C127" t="n">
+        <v>84</v>
+      </c>
+      <c r="D127" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>19</v>
+      </c>
+      <c r="B128" t="n">
+        <v>21</v>
+      </c>
+      <c r="C128" t="n">
+        <v>79</v>
+      </c>
+      <c r="D128" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>19</v>
+      </c>
+      <c r="B129" t="n">
+        <v>31</v>
+      </c>
+      <c r="C129" t="n">
+        <v>54</v>
+      </c>
+      <c r="D129" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>20</v>
+      </c>
+      <c r="B130" t="n">
+        <v>21</v>
+      </c>
+      <c r="C130" t="n">
+        <v>28</v>
+      </c>
+      <c r="D130" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>12</v>
+      </c>
+      <c r="B131" t="n">
+        <v>32</v>
+      </c>
+      <c r="C131" t="n">
+        <v>29</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>28</v>
+      </c>
+      <c r="B132" t="n">
+        <v>29</v>
+      </c>
+      <c r="C132" t="n">
+        <v>25</v>
+      </c>
+      <c r="D132" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>13</v>
+      </c>
+      <c r="B133" t="n">
+        <v>32</v>
+      </c>
+      <c r="C133" t="n">
+        <v>39</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>4</v>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="n">
+        <v>52</v>
+      </c>
+      <c r="D134" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>15</v>
+      </c>
+      <c r="B135" t="n">
+        <v>31</v>
+      </c>
+      <c r="C135" t="n">
+        <v>79</v>
+      </c>
+      <c r="D135" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>14</v>
+      </c>
+      <c r="B136" t="n">
+        <v>2</v>
+      </c>
+      <c r="C136" t="n">
+        <v>65</v>
+      </c>
+      <c r="D136" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>17</v>
+      </c>
+      <c r="B137" t="n">
+        <v>31</v>
+      </c>
+      <c r="C137" t="n">
+        <v>76</v>
+      </c>
+      <c r="D137" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>10</v>
+      </c>
+      <c r="B138" t="n">
+        <v>21</v>
+      </c>
+      <c r="C138" t="n">
+        <v>32</v>
+      </c>
+      <c r="D138" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>5</v>
+      </c>
+      <c r="B139" t="n">
+        <v>33</v>
+      </c>
+      <c r="C139" t="n">
+        <v>57</v>
+      </c>
+      <c r="D139" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>25</v>
+      </c>
+      <c r="B140" t="n">
+        <v>29</v>
+      </c>
+      <c r="C140" t="n">
+        <v>38</v>
+      </c>
+      <c r="D140" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>6</v>
+      </c>
+      <c r="B141" t="n">
+        <v>33</v>
+      </c>
+      <c r="C141" t="n">
+        <v>29</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>13</v>
+      </c>
+      <c r="B142" t="n">
+        <v>30</v>
+      </c>
+      <c r="C142" t="n">
+        <v>88</v>
+      </c>
+      <c r="D142" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>25</v>
+      </c>
+      <c r="B143" t="n">
+        <v>22</v>
+      </c>
+      <c r="C143" t="n">
+        <v>24</v>
+      </c>
+      <c r="D143" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>27</v>
+      </c>
+      <c r="B144" t="n">
+        <v>33</v>
+      </c>
+      <c r="C144" t="n">
+        <v>61</v>
+      </c>
+      <c r="D144" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>15</v>
+      </c>
+      <c r="B145" t="n">
+        <v>22</v>
+      </c>
+      <c r="C145" t="n">
+        <v>34</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>27</v>
+      </c>
+      <c r="B146" t="n">
+        <v>32</v>
+      </c>
+      <c r="C146" t="n">
+        <v>79</v>
+      </c>
+      <c r="D146" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>5</v>
+      </c>
+      <c r="B147" t="n">
+        <v>22</v>
+      </c>
+      <c r="C147" t="n">
+        <v>40</v>
+      </c>
+      <c r="D147" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>8</v>
+      </c>
+      <c r="B148" t="n">
+        <v>33</v>
+      </c>
+      <c r="C148" t="n">
+        <v>71</v>
+      </c>
+      <c r="D148" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>12</v>
+      </c>
+      <c r="B149" t="n">
+        <v>31</v>
+      </c>
+      <c r="C149" t="n">
+        <v>85</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>16</v>
+      </c>
+      <c r="B150" t="n">
+        <v>29</v>
+      </c>
+      <c r="C150" t="n">
+        <v>48</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>14</v>
+      </c>
+      <c r="B151" t="n">
+        <v>22</v>
+      </c>
+      <c r="C151" t="n">
+        <v>62</v>
+      </c>
+      <c r="D151" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>20</v>
+      </c>
+      <c r="B152" t="n">
+        <v>30</v>
+      </c>
+      <c r="C152" t="n">
+        <v>85</v>
+      </c>
+      <c r="D152" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>6</v>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="n">
+        <v>58</v>
+      </c>
+      <c r="D153" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>18</v>
+      </c>
+      <c r="B154" t="n">
+        <v>32</v>
+      </c>
+      <c r="C154" t="n">
+        <v>31</v>
+      </c>
+      <c r="D154" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>4</v>
+      </c>
+      <c r="B155" t="n">
+        <v>29</v>
+      </c>
+      <c r="C155" t="n">
+        <v>35</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>3</v>
+      </c>
+      <c r="B156" t="n">
+        <v>23</v>
+      </c>
+      <c r="C156" t="n">
+        <v>40</v>
+      </c>
+      <c r="D156" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>5</v>
+      </c>
+      <c r="B157" t="n">
+        <v>22</v>
+      </c>
+      <c r="C157" t="n">
+        <v>70</v>
+      </c>
+      <c r="D157" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>3</v>
+      </c>
+      <c r="B158" t="n">
+        <v>33</v>
+      </c>
+      <c r="C158" t="n">
+        <v>24</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>19</v>
+      </c>
+      <c r="B159" t="n">
+        <v>24</v>
+      </c>
+      <c r="C159" t="n">
+        <v>45</v>
+      </c>
+      <c r="D159" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>5</v>
+      </c>
+      <c r="B160" t="n">
+        <v>22</v>
+      </c>
+      <c r="C160" t="n">
+        <v>90</v>
+      </c>
+      <c r="D160" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>28</v>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+      <c r="C161" t="n">
+        <v>87</v>
+      </c>
+      <c r="D161" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>11</v>
+      </c>
+      <c r="B162" t="n">
+        <v>29</v>
+      </c>
+      <c r="C162" t="n">
+        <v>39</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>11</v>
+      </c>
+      <c r="B163" t="n">
+        <v>30</v>
+      </c>
+      <c r="C163" t="n">
+        <v>45</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>9</v>
+      </c>
+      <c r="B164" t="n">
+        <v>24</v>
+      </c>
+      <c r="C164" t="n">
+        <v>77</v>
+      </c>
+      <c r="D164" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>5</v>
+      </c>
+      <c r="B165" t="n">
+        <v>24</v>
+      </c>
+      <c r="C165" t="n">
+        <v>48</v>
+      </c>
+      <c r="D165" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>10</v>
+      </c>
+      <c r="B166" t="n">
+        <v>33</v>
+      </c>
+      <c r="C166" t="n">
+        <v>35</v>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>18</v>
+      </c>
+      <c r="B167" t="n">
+        <v>33</v>
+      </c>
+      <c r="C167" t="n">
+        <v>31</v>
+      </c>
+      <c r="D167" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>5</v>
+      </c>
+      <c r="B168" t="n">
+        <v>31</v>
+      </c>
+      <c r="C168" t="n">
+        <v>82</v>
+      </c>
+      <c r="D168" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>28</v>
+      </c>
+      <c r="B169" t="n">
+        <v>31</v>
+      </c>
+      <c r="C169" t="n">
+        <v>49</v>
+      </c>
+      <c r="D169" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>14</v>
+      </c>
+      <c r="B170" t="n">
+        <v>32</v>
+      </c>
+      <c r="C170" t="n">
+        <v>50</v>
+      </c>
+      <c r="D170" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>5</v>
+      </c>
+      <c r="B171" t="n">
+        <v>33</v>
+      </c>
+      <c r="C171" t="n">
+        <v>52</v>
+      </c>
+      <c r="D171" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>27</v>
+      </c>
+      <c r="B172" t="n">
+        <v>29</v>
+      </c>
+      <c r="C172" t="n">
+        <v>69</v>
+      </c>
+      <c r="D172" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>14</v>
+      </c>
+      <c r="B173" t="n">
+        <v>2</v>
+      </c>
+      <c r="C173" t="n">
+        <v>34</v>
+      </c>
+      <c r="D173" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>11</v>
+      </c>
+      <c r="B174" t="n">
+        <v>32</v>
+      </c>
+      <c r="C174" t="n">
+        <v>44</v>
+      </c>
+      <c r="D174" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>15</v>
+      </c>
+      <c r="B175" t="n">
+        <v>1</v>
+      </c>
+      <c r="C175" t="n">
+        <v>51</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>6</v>
+      </c>
+      <c r="B176" t="n">
+        <v>1</v>
+      </c>
+      <c r="C176" t="n">
+        <v>37</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>8</v>
+      </c>
+      <c r="B177" t="n">
+        <v>33</v>
+      </c>
+      <c r="C177" t="n">
+        <v>23</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>19</v>
+      </c>
+      <c r="B178" t="n">
+        <v>33</v>
+      </c>
+      <c r="C178" t="n">
+        <v>49</v>
+      </c>
+      <c r="D178" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>8</v>
+      </c>
+      <c r="B179" t="n">
+        <v>2</v>
+      </c>
+      <c r="C179" t="n">
+        <v>53</v>
+      </c>
+      <c r="D179" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>14</v>
+      </c>
+      <c r="B180" t="n">
+        <v>2</v>
+      </c>
+      <c r="C180" t="n">
+        <v>51</v>
+      </c>
+      <c r="D180" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>17</v>
+      </c>
+      <c r="B181" t="n">
+        <v>24</v>
+      </c>
+      <c r="C181" t="n">
+        <v>45</v>
+      </c>
+      <c r="D181" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>25</v>
+      </c>
+      <c r="B182" t="n">
+        <v>23</v>
+      </c>
+      <c r="C182" t="n">
+        <v>34</v>
+      </c>
+      <c r="D182" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>15</v>
+      </c>
+      <c r="B183" t="n">
+        <v>29</v>
+      </c>
+      <c r="C183" t="n">
+        <v>49</v>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>13</v>
+      </c>
+      <c r="B184" t="n">
+        <v>32</v>
+      </c>
+      <c r="C184" t="n">
+        <v>69</v>
+      </c>
+      <c r="D184" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>8</v>
+      </c>
+      <c r="B185" t="n">
+        <v>23</v>
+      </c>
+      <c r="C185" t="n">
+        <v>88</v>
+      </c>
+      <c r="D185" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>8</v>
+      </c>
+      <c r="B186" t="n">
+        <v>33</v>
+      </c>
+      <c r="C186" t="n">
+        <v>51</v>
+      </c>
+      <c r="D186" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>18</v>
+      </c>
+      <c r="B187" t="n">
+        <v>23</v>
+      </c>
+      <c r="C187" t="n">
+        <v>63</v>
+      </c>
+      <c r="D187" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>27</v>
+      </c>
+      <c r="B188" t="n">
+        <v>29</v>
+      </c>
+      <c r="C188" t="n">
+        <v>59</v>
+      </c>
+      <c r="D188" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>19</v>
+      </c>
+      <c r="B189" t="n">
+        <v>30</v>
+      </c>
+      <c r="C189" t="n">
+        <v>53</v>
+      </c>
+      <c r="D189" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>15</v>
+      </c>
+      <c r="B190" t="n">
+        <v>29</v>
+      </c>
+      <c r="C190" t="n">
+        <v>77</v>
+      </c>
+      <c r="D190" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>18</v>
+      </c>
+      <c r="B191" t="n">
+        <v>21</v>
+      </c>
+      <c r="C191" t="n">
+        <v>38</v>
+      </c>
+      <c r="D191" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>27</v>
+      </c>
+      <c r="B192" t="n">
+        <v>30</v>
+      </c>
+      <c r="C192" t="n">
+        <v>40</v>
+      </c>
+      <c r="D192" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>3</v>
+      </c>
+      <c r="B193" t="n">
+        <v>23</v>
+      </c>
+      <c r="C193" t="n">
+        <v>53</v>
+      </c>
+      <c r="D193" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>27</v>
+      </c>
+      <c r="B194" t="n">
+        <v>29</v>
+      </c>
+      <c r="C194" t="n">
+        <v>24</v>
+      </c>
+      <c r="D194" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>4</v>
+      </c>
+      <c r="B195" t="n">
+        <v>33</v>
+      </c>
+      <c r="C195" t="n">
+        <v>59</v>
+      </c>
+      <c r="D195" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>9</v>
+      </c>
+      <c r="B196" t="n">
+        <v>23</v>
+      </c>
+      <c r="C196" t="n">
+        <v>50</v>
+      </c>
+      <c r="D196" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>3</v>
+      </c>
+      <c r="B197" t="n">
+        <v>31</v>
+      </c>
+      <c r="C197" t="n">
+        <v>89</v>
+      </c>
+      <c r="D197" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>8</v>
+      </c>
+      <c r="B198" t="n">
+        <v>2</v>
+      </c>
+      <c r="C198" t="n">
+        <v>27</v>
+      </c>
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>11</v>
+      </c>
+      <c r="B199" t="n">
+        <v>2</v>
+      </c>
+      <c r="C199" t="n">
+        <v>23</v>
+      </c>
+      <c r="D199" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>15</v>
+      </c>
+      <c r="B200" t="n">
+        <v>33</v>
+      </c>
+      <c r="C200" t="n">
+        <v>65</v>
+      </c>
+      <c r="D200" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>7</v>
+      </c>
+      <c r="B201" t="n">
+        <v>2</v>
+      </c>
+      <c r="C201" t="n">
+        <v>60</v>
+      </c>
+      <c r="D201" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>27</v>
+      </c>
+      <c r="B202" t="n">
+        <v>2</v>
+      </c>
+      <c r="C202" t="n">
+        <v>40</v>
+      </c>
+      <c r="D202" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>14</v>
+      </c>
+      <c r="B203" t="n">
+        <v>30</v>
+      </c>
+      <c r="C203" t="n">
+        <v>76</v>
+      </c>
+      <c r="D203" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>7</v>
+      </c>
+      <c r="B204" t="n">
+        <v>32</v>
+      </c>
+      <c r="C204" t="n">
+        <v>52</v>
+      </c>
+      <c r="D204" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>25</v>
+      </c>
+      <c r="B205" t="n">
+        <v>24</v>
+      </c>
+      <c r="C205" t="n">
+        <v>33</v>
+      </c>
+      <c r="D205" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>4</v>
+      </c>
+      <c r="B206" t="n">
+        <v>29</v>
+      </c>
+      <c r="C206" t="n">
+        <v>89</v>
+      </c>
+      <c r="D206" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>4</v>
+      </c>
+      <c r="B207" t="n">
+        <v>33</v>
+      </c>
+      <c r="C207" t="n">
+        <v>88</v>
+      </c>
+      <c r="D207" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>15</v>
+      </c>
+      <c r="B208" t="n">
+        <v>33</v>
+      </c>
+      <c r="C208" t="n">
+        <v>31</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>20</v>
+      </c>
+      <c r="B209" t="n">
+        <v>24</v>
+      </c>
+      <c r="C209" t="n">
+        <v>52</v>
+      </c>
+      <c r="D209" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>20</v>
+      </c>
+      <c r="B210" t="n">
+        <v>32</v>
+      </c>
+      <c r="C210" t="n">
+        <v>90</v>
+      </c>
+      <c r="D210" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>17</v>
+      </c>
+      <c r="B211" t="n">
+        <v>2</v>
+      </c>
+      <c r="C211" t="n">
+        <v>48</v>
+      </c>
+      <c r="D211" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>15</v>
+      </c>
+      <c r="B212" t="n">
+        <v>30</v>
+      </c>
+      <c r="C212" t="n">
+        <v>42</v>
+      </c>
+      <c r="D212" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>15</v>
+      </c>
+      <c r="B213" t="n">
+        <v>31</v>
+      </c>
+      <c r="C213" t="n">
+        <v>73</v>
+      </c>
+      <c r="D213" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>12</v>
+      </c>
+      <c r="B214" t="n">
+        <v>31</v>
+      </c>
+      <c r="C214" t="n">
+        <v>51</v>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2257,4 +4196,31 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Data Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>COUNTA(data!A:A)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>